<commit_message>
feat: reading csv and checking all customer TINs in a row
</commit_message>
<xml_diff>
--- a/data/TIN_database/example.xlsx
+++ b/data/TIN_database/example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\palot\Documents\42\AI project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\zpalotas\projects\AI project\github\data\TIN_database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{59D96203-337A-4817-9F98-2A88DAAC0AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8B0BFB4-C048-4950-8357-4052A9F4CC16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{043BCBC4-A84C-40C5-8A84-B441781113F4}"/>
   </bookViews>
@@ -53,56 +53,56 @@
     <t>Max Mustermann</t>
   </si>
   <si>
-    <t>John Doe</t>
-  </si>
-  <si>
     <t>Maria Musterfrau</t>
   </si>
   <si>
-    <t>Maija Meikäläinen </t>
-  </si>
-  <si>
-    <t>FI</t>
-  </si>
-  <si>
     <t>Country_code</t>
   </si>
   <si>
     <t>DE</t>
   </si>
   <si>
-    <t>UK</t>
-  </si>
-  <si>
     <t>AT</t>
   </si>
   <si>
     <t>Germany</t>
   </si>
   <si>
-    <t>United Kingdom</t>
-  </si>
-  <si>
     <t>Austria</t>
   </si>
   <si>
-    <t>Finland</t>
-  </si>
-  <si>
-    <t>Teszt Elek</t>
-  </si>
-  <si>
-    <t>Hungary</t>
-  </si>
-  <si>
-    <t>HU</t>
+    <t>12-345/6789</t>
+  </si>
+  <si>
+    <t>Brunei</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>BN</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>Test Tester</t>
+  </si>
+  <si>
+    <t>Some Body</t>
+  </si>
+  <si>
+    <t>C99999999999999999</t>
+  </si>
+  <si>
+    <t>29-999999</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -110,13 +110,6 @@
       <family val="2"/>
       <charset val="238"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF0A0A0A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -139,9 +132,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,13 +468,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EF01132-D9CD-4BF3-9788-B089A94CB751}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="1" max="1" width="18.69921875" customWidth="1"/>
+    <col min="4" max="4" width="9.8984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -490,7 +483,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -499,59 +492,60 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>123456789</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s">
-        <v>11</v>
+      <c r="D4" t="s">
+        <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="D5" t="s">
         <v>18</v>
-      </c>
-      <c r="C6" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>